<commit_message>
Update DU4 for 2026, including housing addition
</commit_message>
<xml_diff>
--- a/data/6484.0/648401.xlsx
+++ b/data/6484.0/648401.xlsx
@@ -17,221 +17,221 @@
     <sheet name="Enquiries" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="A128473239F">Data1!$AC$1:$AC$10,Data1!$AC$11:$AC$105</definedName>
-    <definedName name="A128473239F_Data">Data1!$AC$11:$AC$105</definedName>
-    <definedName name="A128473239F_Latest">Data1!$AC$105</definedName>
-    <definedName name="A128473240R">Data1!$BL$1:$BL$10,Data1!$BL$23:$BL$105</definedName>
-    <definedName name="A128473240R_Data">Data1!$BL$23:$BL$105</definedName>
-    <definedName name="A128473240R_Latest">Data1!$BL$105</definedName>
-    <definedName name="A128473315W">Data1!$U$1:$U$10,Data1!$U$11:$U$105</definedName>
-    <definedName name="A128473315W_Data">Data1!$U$11:$U$105</definedName>
-    <definedName name="A128473315W_Latest">Data1!$U$105</definedName>
-    <definedName name="A128473316X">Data1!$BD$1:$BD$10,Data1!$BD$23:$BD$105</definedName>
-    <definedName name="A128473316X_Data">Data1!$BD$23:$BD$105</definedName>
-    <definedName name="A128473316X_Latest">Data1!$BD$105</definedName>
-    <definedName name="A128473361K">Data1!$AA$1:$AA$10,Data1!$AA$11:$AA$105</definedName>
-    <definedName name="A128473361K_Data">Data1!$AA$11:$AA$105</definedName>
-    <definedName name="A128473361K_Latest">Data1!$AA$105</definedName>
-    <definedName name="A128473362L">Data1!$BJ$1:$BJ$10,Data1!$BJ$23:$BJ$105</definedName>
-    <definedName name="A128473362L_Data">Data1!$BJ$23:$BJ$105</definedName>
-    <definedName name="A128473362L_Latest">Data1!$BJ$105</definedName>
-    <definedName name="A128473449C">Data1!$P$1:$P$10,Data1!$P$11:$P$105</definedName>
-    <definedName name="A128473449C_Data">Data1!$P$11:$P$105</definedName>
-    <definedName name="A128473449C_Latest">Data1!$P$105</definedName>
-    <definedName name="A128473450L">Data1!$AY$1:$AY$10,Data1!$AY$23:$AY$105</definedName>
-    <definedName name="A128473450L_Data">Data1!$AY$23:$AY$105</definedName>
-    <definedName name="A128473450L_Latest">Data1!$AY$105</definedName>
-    <definedName name="A128473623X">Data1!$I$1:$I$10,Data1!$I$11:$I$105</definedName>
-    <definedName name="A128473623X_Data">Data1!$I$11:$I$105</definedName>
-    <definedName name="A128473623X_Latest">Data1!$I$105</definedName>
-    <definedName name="A128473624A">Data1!$AR$1:$AR$10,Data1!$AR$23:$AR$105</definedName>
-    <definedName name="A128473624A_Data">Data1!$AR$23:$AR$105</definedName>
-    <definedName name="A128473624A_Latest">Data1!$AR$105</definedName>
-    <definedName name="A128474303F">Data1!$R$1:$R$10,Data1!$R$11:$R$105</definedName>
-    <definedName name="A128474303F_Data">Data1!$R$11:$R$105</definedName>
-    <definedName name="A128474303F_Latest">Data1!$R$105</definedName>
-    <definedName name="A128474304J">Data1!$BA$1:$BA$10,Data1!$BA$23:$BA$105</definedName>
-    <definedName name="A128474304J_Data">Data1!$BA$23:$BA$105</definedName>
-    <definedName name="A128474304J_Latest">Data1!$BA$105</definedName>
-    <definedName name="A128475063X">Data1!$X$1:$X$10,Data1!$X$11:$X$105</definedName>
-    <definedName name="A128475063X_Data">Data1!$X$11:$X$105</definedName>
-    <definedName name="A128475063X_Latest">Data1!$X$105</definedName>
-    <definedName name="A128475064A">Data1!$BG$1:$BG$10,Data1!$BG$23:$BG$105</definedName>
-    <definedName name="A128475064A_Data">Data1!$BG$23:$BG$105</definedName>
-    <definedName name="A128475064A_Latest">Data1!$BG$105</definedName>
-    <definedName name="A128475329W">Data1!$H$1:$H$10,Data1!$H$11:$H$105</definedName>
-    <definedName name="A128475329W_Data">Data1!$H$11:$H$105</definedName>
-    <definedName name="A128475329W_Latest">Data1!$H$105</definedName>
-    <definedName name="A128475330F">Data1!$AQ$1:$AQ$10,Data1!$AQ$23:$AQ$105</definedName>
-    <definedName name="A128475330F_Data">Data1!$AQ$23:$AQ$105</definedName>
-    <definedName name="A128475330F_Latest">Data1!$AQ$105</definedName>
-    <definedName name="A128475405L">Data1!$Q$1:$Q$10,Data1!$Q$11:$Q$105</definedName>
-    <definedName name="A128475405L_Data">Data1!$Q$11:$Q$105</definedName>
-    <definedName name="A128475405L_Latest">Data1!$Q$105</definedName>
-    <definedName name="A128475406R">Data1!$AZ$1:$AZ$10,Data1!$AZ$23:$AZ$105</definedName>
-    <definedName name="A128475406R_Data">Data1!$AZ$23:$AZ$105</definedName>
-    <definedName name="A128475406R_Latest">Data1!$AZ$105</definedName>
-    <definedName name="A128475583C">Data1!$M$1:$M$10,Data1!$M$11:$M$105</definedName>
-    <definedName name="A128475583C_Data">Data1!$M$11:$M$105</definedName>
-    <definedName name="A128475583C_Latest">Data1!$M$105</definedName>
-    <definedName name="A128475584F">Data1!$AV$1:$AV$10,Data1!$AV$23:$AV$105</definedName>
-    <definedName name="A128475584F_Data">Data1!$AV$23:$AV$105</definedName>
-    <definedName name="A128475584F_Latest">Data1!$AV$105</definedName>
-    <definedName name="A128475629X">Data1!$D$1:$D$10,Data1!$D$11:$D$105</definedName>
-    <definedName name="A128475629X_Data">Data1!$D$11:$D$105</definedName>
-    <definedName name="A128475629X_Latest">Data1!$D$105</definedName>
-    <definedName name="A128475630J">Data1!$AM$1:$AM$10,Data1!$AM$23:$AM$105</definedName>
-    <definedName name="A128475630J_Data">Data1!$AM$23:$AM$105</definedName>
-    <definedName name="A128475630J_Latest">Data1!$AM$105</definedName>
-    <definedName name="A128475797K">Data1!$Z$1:$Z$10,Data1!$Z$11:$Z$105</definedName>
-    <definedName name="A128475797K_Data">Data1!$Z$11:$Z$105</definedName>
-    <definedName name="A128475797K_Latest">Data1!$Z$105</definedName>
-    <definedName name="A128475798L">Data1!$BI$1:$BI$10,Data1!$BI$23:$BI$105</definedName>
-    <definedName name="A128475798L_Data">Data1!$BI$23:$BI$105</definedName>
-    <definedName name="A128475798L_Latest">Data1!$BI$105</definedName>
-    <definedName name="A128476505R">Data1!$AI$1:$AI$10,Data1!$AI$11:$AI$105</definedName>
-    <definedName name="A128476505R_Data">Data1!$AI$11:$AI$105</definedName>
-    <definedName name="A128476505R_Latest">Data1!$AI$105</definedName>
-    <definedName name="A128476506T">Data1!$BS$1:$BS$10,Data1!$BS$23:$BS$105</definedName>
-    <definedName name="A128476506T_Data">Data1!$BS$23:$BS$105</definedName>
-    <definedName name="A128476506T_Latest">Data1!$BS$105</definedName>
-    <definedName name="A128476849V">Data1!$S$1:$S$10,Data1!$S$11:$S$105</definedName>
-    <definedName name="A128476849V_Data">Data1!$S$11:$S$105</definedName>
-    <definedName name="A128476849V_Latest">Data1!$S$105</definedName>
-    <definedName name="A128476850C">Data1!$BB$1:$BB$10,Data1!$BB$23:$BB$105</definedName>
-    <definedName name="A128476850C_Data">Data1!$BB$23:$BB$105</definedName>
-    <definedName name="A128476850C_Latest">Data1!$BB$105</definedName>
-    <definedName name="A128477043A">Data1!$AB$1:$AB$10,Data1!$AB$11:$AB$105</definedName>
-    <definedName name="A128477043A_Data">Data1!$AB$11:$AB$105</definedName>
-    <definedName name="A128477043A_Latest">Data1!$AB$105</definedName>
-    <definedName name="A128477044C">Data1!$BK$1:$BK$10,Data1!$BK$23:$BK$105</definedName>
-    <definedName name="A128477044C_Data">Data1!$BK$23:$BK$105</definedName>
-    <definedName name="A128477044C_Latest">Data1!$BK$105</definedName>
-    <definedName name="A128477399R">Data1!$J$1:$J$10,Data1!$J$11:$J$105</definedName>
-    <definedName name="A128477399R_Data">Data1!$J$11:$J$105</definedName>
-    <definedName name="A128477399R_Latest">Data1!$J$105</definedName>
-    <definedName name="A128477400L">Data1!$AS$1:$AS$10,Data1!$AS$23:$AS$105</definedName>
-    <definedName name="A128477400L_Data">Data1!$AS$23:$AS$105</definedName>
-    <definedName name="A128477400L_Latest">Data1!$AS$105</definedName>
-    <definedName name="A128477405X">Data1!$F$1:$F$10,Data1!$F$11:$F$105</definedName>
-    <definedName name="A128477405X_Data">Data1!$F$11:$F$105</definedName>
-    <definedName name="A128477405X_Latest">Data1!$F$105</definedName>
-    <definedName name="A128477406A">Data1!$AO$1:$AO$10,Data1!$AO$23:$AO$105</definedName>
-    <definedName name="A128477406A_Data">Data1!$AO$23:$AO$105</definedName>
-    <definedName name="A128477406A_Latest">Data1!$AO$105</definedName>
-    <definedName name="A128478317T">Data1!$B$1:$B$10,Data1!$B$11:$B$105</definedName>
-    <definedName name="A128478317T_Data">Data1!$B$11:$B$105</definedName>
-    <definedName name="A128478317T_Latest">Data1!$B$105</definedName>
-    <definedName name="A128478318V">Data1!$AK$1:$AK$10,Data1!$AK$23:$AK$105</definedName>
-    <definedName name="A128478318V_Data">Data1!$AK$23:$AK$105</definedName>
-    <definedName name="A128478318V_Latest">Data1!$AK$105</definedName>
-    <definedName name="A128478473V">Data1!$Y$1:$Y$10,Data1!$Y$11:$Y$105</definedName>
-    <definedName name="A128478473V_Data">Data1!$Y$11:$Y$105</definedName>
-    <definedName name="A128478473V_Latest">Data1!$Y$105</definedName>
-    <definedName name="A128478474W">Data1!$BH$1:$BH$10,Data1!$BH$23:$BH$105</definedName>
-    <definedName name="A128478474W_Data">Data1!$BH$23:$BH$105</definedName>
-    <definedName name="A128478474W_Latest">Data1!$BH$105</definedName>
-    <definedName name="A128478847A">Data1!$N$1:$N$10,Data1!$N$11:$N$105</definedName>
-    <definedName name="A128478847A_Data">Data1!$N$11:$N$105</definedName>
-    <definedName name="A128478847A_Latest">Data1!$N$105</definedName>
-    <definedName name="A128478848C">Data1!$AW$1:$AW$10,Data1!$AW$23:$AW$105</definedName>
-    <definedName name="A128478848C_Data">Data1!$AW$23:$AW$105</definedName>
-    <definedName name="A128478848C_Latest">Data1!$AW$105</definedName>
-    <definedName name="A128479215W">Data1!$E$1:$E$10,Data1!$E$11:$E$105</definedName>
-    <definedName name="A128479215W_Data">Data1!$E$11:$E$105</definedName>
-    <definedName name="A128479215W_Latest">Data1!$E$105</definedName>
-    <definedName name="A128479216X">Data1!$AN$1:$AN$10,Data1!$AN$23:$AN$105</definedName>
-    <definedName name="A128479216X_Data">Data1!$AN$23:$AN$105</definedName>
-    <definedName name="A128479216X_Latest">Data1!$AN$105</definedName>
-    <definedName name="A128479281V">Data1!$K$1:$K$10,Data1!$K$11:$K$105</definedName>
-    <definedName name="A128479281V_Data">Data1!$K$11:$K$105</definedName>
-    <definedName name="A128479281V_Latest">Data1!$K$105</definedName>
-    <definedName name="A128479282W">Data1!$AT$1:$AT$10,Data1!$AT$23:$AT$105</definedName>
-    <definedName name="A128479282W_Data">Data1!$AT$23:$AT$105</definedName>
-    <definedName name="A128479282W_Latest">Data1!$AT$105</definedName>
-    <definedName name="A128480133R">Data1!$AJ$1:$AJ$10,Data1!$AJ$11:$AJ$105</definedName>
-    <definedName name="A128480133R_Data">Data1!$AJ$11:$AJ$105</definedName>
-    <definedName name="A128480133R_Latest">Data1!$AJ$105</definedName>
-    <definedName name="A128480134T">Data1!$BT$1:$BT$10,Data1!$BT$23:$BT$105</definedName>
-    <definedName name="A128480134T_Data">Data1!$BT$23:$BT$105</definedName>
-    <definedName name="A128480134T_Latest">Data1!$BT$105</definedName>
-    <definedName name="A128480215V">Data1!$G$1:$G$10,Data1!$G$11:$G$105</definedName>
-    <definedName name="A128480215V_Data">Data1!$G$11:$G$105</definedName>
-    <definedName name="A128480215V_Latest">Data1!$G$105</definedName>
-    <definedName name="A128480216W">Data1!$AP$1:$AP$10,Data1!$AP$23:$AP$105</definedName>
-    <definedName name="A128480216W_Data">Data1!$AP$23:$AP$105</definedName>
-    <definedName name="A128480216W_Latest">Data1!$AP$105</definedName>
-    <definedName name="A128480733V">Data1!$C$1:$C$10,Data1!$C$11:$C$105</definedName>
-    <definedName name="A128480733V_Data">Data1!$C$11:$C$105</definedName>
-    <definedName name="A128480733V_Latest">Data1!$C$105</definedName>
-    <definedName name="A128480734W">Data1!$AL$1:$AL$10,Data1!$AL$23:$AL$105</definedName>
-    <definedName name="A128480734W_Data">Data1!$AL$23:$AL$105</definedName>
-    <definedName name="A128480734W_Latest">Data1!$AL$105</definedName>
-    <definedName name="A128481587A">Data1!$AD$1:$AD$10,Data1!$AD$11:$AD$105</definedName>
-    <definedName name="A128481587A_Data">Data1!$AD$11:$AD$105</definedName>
-    <definedName name="A128481587A_Latest">Data1!$AD$105</definedName>
-    <definedName name="A128481588C">Data1!$BM$1:$BM$10,Data1!$BM$23:$BM$105</definedName>
-    <definedName name="A128481588C_Data">Data1!$BM$23:$BM$105</definedName>
-    <definedName name="A128481588C_Latest">Data1!$BM$105</definedName>
-    <definedName name="A128481639T">Data1!$AH$1:$AH$10,Data1!$AH$11:$AH$105</definedName>
-    <definedName name="A128481639T_Data">Data1!$AH$11:$AH$105</definedName>
-    <definedName name="A128481639T_Latest">Data1!$AH$105</definedName>
-    <definedName name="A128481640A">Data1!$BR$1:$BR$10,Data1!$BR$23:$BR$105</definedName>
-    <definedName name="A128481640A_Data">Data1!$BR$23:$BR$105</definedName>
-    <definedName name="A128481640A_Latest">Data1!$BR$105</definedName>
-    <definedName name="A128482435J">Data1!$V$1:$V$10,Data1!$V$11:$V$105</definedName>
-    <definedName name="A128482435J_Data">Data1!$V$11:$V$105</definedName>
-    <definedName name="A128482435J_Latest">Data1!$V$105</definedName>
-    <definedName name="A128482436K">Data1!$BE$1:$BE$10,Data1!$BE$23:$BE$105</definedName>
-    <definedName name="A128482436K_Data">Data1!$BE$23:$BE$105</definedName>
-    <definedName name="A128482436K_Latest">Data1!$BE$105</definedName>
-    <definedName name="A128483461F">Data1!$AG$1:$AG$10,Data1!$AG$11:$AG$105</definedName>
-    <definedName name="A128483461F_Data">Data1!$AG$11:$AG$105</definedName>
-    <definedName name="A128483461F_Latest">Data1!$AG$105</definedName>
-    <definedName name="A128483462J">Data1!$BQ$1:$BQ$10,Data1!$BQ$23:$BQ$105</definedName>
-    <definedName name="A128483462J_Data">Data1!$BQ$23:$BQ$105</definedName>
-    <definedName name="A128483462J_Latest">Data1!$BQ$105</definedName>
-    <definedName name="A128484257R">Data1!$L$1:$L$10,Data1!$L$11:$L$105</definedName>
-    <definedName name="A128484257R_Data">Data1!$L$11:$L$105</definedName>
-    <definedName name="A128484257R_Latest">Data1!$L$105</definedName>
-    <definedName name="A128484258T">Data1!$AU$1:$AU$10,Data1!$AU$23:$AU$105</definedName>
-    <definedName name="A128484258T_Data">Data1!$AU$23:$AU$105</definedName>
-    <definedName name="A128484258T_Latest">Data1!$AU$105</definedName>
-    <definedName name="A128484685K">Data1!$W$1:$W$10,Data1!$W$11:$W$105</definedName>
-    <definedName name="A128484685K_Data">Data1!$W$11:$W$105</definedName>
-    <definedName name="A128484685K_Latest">Data1!$W$105</definedName>
-    <definedName name="A128484686L">Data1!$BF$1:$BF$10,Data1!$BF$23:$BF$105</definedName>
-    <definedName name="A128484686L_Data">Data1!$BF$23:$BF$105</definedName>
-    <definedName name="A128484686L_Latest">Data1!$BF$105</definedName>
-    <definedName name="A128485865L">Data1!$O$1:$O$10,Data1!$O$11:$O$105</definedName>
-    <definedName name="A128485865L_Data">Data1!$O$11:$O$105</definedName>
-    <definedName name="A128485865L_Latest">Data1!$O$105</definedName>
-    <definedName name="A128485866R">Data1!$AX$1:$AX$10,Data1!$AX$23:$AX$105</definedName>
-    <definedName name="A128485866R_Data">Data1!$AX$23:$AX$105</definedName>
-    <definedName name="A128485866R_Latest">Data1!$AX$105</definedName>
-    <definedName name="A128485881L">Data1!$T$1:$T$10,Data1!$T$11:$T$105</definedName>
-    <definedName name="A128485881L_Data">Data1!$T$11:$T$105</definedName>
-    <definedName name="A128485881L_Latest">Data1!$T$105</definedName>
-    <definedName name="A128485882R">Data1!$BC$1:$BC$10,Data1!$BC$23:$BC$105</definedName>
-    <definedName name="A128485882R_Data">Data1!$BC$23:$BC$105</definedName>
-    <definedName name="A128485882R_Latest">Data1!$BC$105</definedName>
-    <definedName name="A130184496J">Data1!$BN$1:$BN$10,Data1!$BN$23:$BN$105</definedName>
-    <definedName name="A130184496J_Data">Data1!$BN$23:$BN$105</definedName>
-    <definedName name="A130184496J_Latest">Data1!$BN$105</definedName>
-    <definedName name="A130184497K">Data1!$BP$1:$BP$10,Data1!$BP$23:$BP$105</definedName>
-    <definedName name="A130184497K_Data">Data1!$BP$23:$BP$105</definedName>
-    <definedName name="A130184497K_Latest">Data1!$BP$105</definedName>
-    <definedName name="A130184498L">Data1!$BO$1:$BO$10,Data1!$BO$23:$BO$105</definedName>
-    <definedName name="A130184498L_Data">Data1!$BO$23:$BO$105</definedName>
-    <definedName name="A130184498L_Latest">Data1!$BO$105</definedName>
-    <definedName name="A130184499R">Data1!$AE$1:$AE$10,Data1!$AE$11:$AE$105</definedName>
-    <definedName name="A130184499R_Data">Data1!$AE$11:$AE$105</definedName>
-    <definedName name="A130184499R_Latest">Data1!$AE$105</definedName>
-    <definedName name="A130184501R">Data1!$AF$1:$AF$10,Data1!$AF$11:$AF$105</definedName>
-    <definedName name="A130184501R_Data">Data1!$AF$11:$AF$105</definedName>
-    <definedName name="A130184501R_Latest">Data1!$AF$105</definedName>
-    <definedName name="Date_Range">Data1!$A$2:$A$10,Data1!$A$11:$A$105</definedName>
-    <definedName name="Date_Range_Data">Data1!$A$11:$A$105</definedName>
+    <definedName name="A128473239F">Data1!$AC$1:$AC$10,Data1!$AC$11:$AC$107</definedName>
+    <definedName name="A128473239F_Data">Data1!$AC$11:$AC$107</definedName>
+    <definedName name="A128473239F_Latest">Data1!$AC$107</definedName>
+    <definedName name="A128473240R">Data1!$BL$1:$BL$10,Data1!$BL$23:$BL$107</definedName>
+    <definedName name="A128473240R_Data">Data1!$BL$23:$BL$107</definedName>
+    <definedName name="A128473240R_Latest">Data1!$BL$107</definedName>
+    <definedName name="A128473315W">Data1!$U$1:$U$10,Data1!$U$11:$U$107</definedName>
+    <definedName name="A128473315W_Data">Data1!$U$11:$U$107</definedName>
+    <definedName name="A128473315W_Latest">Data1!$U$107</definedName>
+    <definedName name="A128473316X">Data1!$BD$1:$BD$10,Data1!$BD$23:$BD$107</definedName>
+    <definedName name="A128473316X_Data">Data1!$BD$23:$BD$107</definedName>
+    <definedName name="A128473316X_Latest">Data1!$BD$107</definedName>
+    <definedName name="A128473361K">Data1!$AA$1:$AA$10,Data1!$AA$11:$AA$107</definedName>
+    <definedName name="A128473361K_Data">Data1!$AA$11:$AA$107</definedName>
+    <definedName name="A128473361K_Latest">Data1!$AA$107</definedName>
+    <definedName name="A128473362L">Data1!$BJ$1:$BJ$10,Data1!$BJ$23:$BJ$107</definedName>
+    <definedName name="A128473362L_Data">Data1!$BJ$23:$BJ$107</definedName>
+    <definedName name="A128473362L_Latest">Data1!$BJ$107</definedName>
+    <definedName name="A128473449C">Data1!$P$1:$P$10,Data1!$P$11:$P$107</definedName>
+    <definedName name="A128473449C_Data">Data1!$P$11:$P$107</definedName>
+    <definedName name="A128473449C_Latest">Data1!$P$107</definedName>
+    <definedName name="A128473450L">Data1!$AY$1:$AY$10,Data1!$AY$23:$AY$107</definedName>
+    <definedName name="A128473450L_Data">Data1!$AY$23:$AY$107</definedName>
+    <definedName name="A128473450L_Latest">Data1!$AY$107</definedName>
+    <definedName name="A128473623X">Data1!$I$1:$I$10,Data1!$I$11:$I$107</definedName>
+    <definedName name="A128473623X_Data">Data1!$I$11:$I$107</definedName>
+    <definedName name="A128473623X_Latest">Data1!$I$107</definedName>
+    <definedName name="A128473624A">Data1!$AR$1:$AR$10,Data1!$AR$23:$AR$107</definedName>
+    <definedName name="A128473624A_Data">Data1!$AR$23:$AR$107</definedName>
+    <definedName name="A128473624A_Latest">Data1!$AR$107</definedName>
+    <definedName name="A128474303F">Data1!$R$1:$R$10,Data1!$R$11:$R$107</definedName>
+    <definedName name="A128474303F_Data">Data1!$R$11:$R$107</definedName>
+    <definedName name="A128474303F_Latest">Data1!$R$107</definedName>
+    <definedName name="A128474304J">Data1!$BA$1:$BA$10,Data1!$BA$23:$BA$107</definedName>
+    <definedName name="A128474304J_Data">Data1!$BA$23:$BA$107</definedName>
+    <definedName name="A128474304J_Latest">Data1!$BA$107</definedName>
+    <definedName name="A128475063X">Data1!$X$1:$X$10,Data1!$X$11:$X$107</definedName>
+    <definedName name="A128475063X_Data">Data1!$X$11:$X$107</definedName>
+    <definedName name="A128475063X_Latest">Data1!$X$107</definedName>
+    <definedName name="A128475064A">Data1!$BG$1:$BG$10,Data1!$BG$23:$BG$107</definedName>
+    <definedName name="A128475064A_Data">Data1!$BG$23:$BG$107</definedName>
+    <definedName name="A128475064A_Latest">Data1!$BG$107</definedName>
+    <definedName name="A128475329W">Data1!$H$1:$H$10,Data1!$H$11:$H$107</definedName>
+    <definedName name="A128475329W_Data">Data1!$H$11:$H$107</definedName>
+    <definedName name="A128475329W_Latest">Data1!$H$107</definedName>
+    <definedName name="A128475330F">Data1!$AQ$1:$AQ$10,Data1!$AQ$23:$AQ$107</definedName>
+    <definedName name="A128475330F_Data">Data1!$AQ$23:$AQ$107</definedName>
+    <definedName name="A128475330F_Latest">Data1!$AQ$107</definedName>
+    <definedName name="A128475405L">Data1!$Q$1:$Q$10,Data1!$Q$11:$Q$107</definedName>
+    <definedName name="A128475405L_Data">Data1!$Q$11:$Q$107</definedName>
+    <definedName name="A128475405L_Latest">Data1!$Q$107</definedName>
+    <definedName name="A128475406R">Data1!$AZ$1:$AZ$10,Data1!$AZ$23:$AZ$107</definedName>
+    <definedName name="A128475406R_Data">Data1!$AZ$23:$AZ$107</definedName>
+    <definedName name="A128475406R_Latest">Data1!$AZ$107</definedName>
+    <definedName name="A128475583C">Data1!$M$1:$M$10,Data1!$M$11:$M$107</definedName>
+    <definedName name="A128475583C_Data">Data1!$M$11:$M$107</definedName>
+    <definedName name="A128475583C_Latest">Data1!$M$107</definedName>
+    <definedName name="A128475584F">Data1!$AV$1:$AV$10,Data1!$AV$23:$AV$107</definedName>
+    <definedName name="A128475584F_Data">Data1!$AV$23:$AV$107</definedName>
+    <definedName name="A128475584F_Latest">Data1!$AV$107</definedName>
+    <definedName name="A128475629X">Data1!$D$1:$D$10,Data1!$D$11:$D$107</definedName>
+    <definedName name="A128475629X_Data">Data1!$D$11:$D$107</definedName>
+    <definedName name="A128475629X_Latest">Data1!$D$107</definedName>
+    <definedName name="A128475630J">Data1!$AM$1:$AM$10,Data1!$AM$23:$AM$107</definedName>
+    <definedName name="A128475630J_Data">Data1!$AM$23:$AM$107</definedName>
+    <definedName name="A128475630J_Latest">Data1!$AM$107</definedName>
+    <definedName name="A128475797K">Data1!$Z$1:$Z$10,Data1!$Z$11:$Z$107</definedName>
+    <definedName name="A128475797K_Data">Data1!$Z$11:$Z$107</definedName>
+    <definedName name="A128475797K_Latest">Data1!$Z$107</definedName>
+    <definedName name="A128475798L">Data1!$BI$1:$BI$10,Data1!$BI$23:$BI$107</definedName>
+    <definedName name="A128475798L_Data">Data1!$BI$23:$BI$107</definedName>
+    <definedName name="A128475798L_Latest">Data1!$BI$107</definedName>
+    <definedName name="A128476505R">Data1!$AI$1:$AI$10,Data1!$AI$11:$AI$107</definedName>
+    <definedName name="A128476505R_Data">Data1!$AI$11:$AI$107</definedName>
+    <definedName name="A128476505R_Latest">Data1!$AI$107</definedName>
+    <definedName name="A128476506T">Data1!$BS$1:$BS$10,Data1!$BS$23:$BS$107</definedName>
+    <definedName name="A128476506T_Data">Data1!$BS$23:$BS$107</definedName>
+    <definedName name="A128476506T_Latest">Data1!$BS$107</definedName>
+    <definedName name="A128476849V">Data1!$S$1:$S$10,Data1!$S$11:$S$107</definedName>
+    <definedName name="A128476849V_Data">Data1!$S$11:$S$107</definedName>
+    <definedName name="A128476849V_Latest">Data1!$S$107</definedName>
+    <definedName name="A128476850C">Data1!$BB$1:$BB$10,Data1!$BB$23:$BB$107</definedName>
+    <definedName name="A128476850C_Data">Data1!$BB$23:$BB$107</definedName>
+    <definedName name="A128476850C_Latest">Data1!$BB$107</definedName>
+    <definedName name="A128477043A">Data1!$AB$1:$AB$10,Data1!$AB$11:$AB$107</definedName>
+    <definedName name="A128477043A_Data">Data1!$AB$11:$AB$107</definedName>
+    <definedName name="A128477043A_Latest">Data1!$AB$107</definedName>
+    <definedName name="A128477044C">Data1!$BK$1:$BK$10,Data1!$BK$23:$BK$107</definedName>
+    <definedName name="A128477044C_Data">Data1!$BK$23:$BK$107</definedName>
+    <definedName name="A128477044C_Latest">Data1!$BK$107</definedName>
+    <definedName name="A128477399R">Data1!$J$1:$J$10,Data1!$J$11:$J$107</definedName>
+    <definedName name="A128477399R_Data">Data1!$J$11:$J$107</definedName>
+    <definedName name="A128477399R_Latest">Data1!$J$107</definedName>
+    <definedName name="A128477400L">Data1!$AS$1:$AS$10,Data1!$AS$23:$AS$107</definedName>
+    <definedName name="A128477400L_Data">Data1!$AS$23:$AS$107</definedName>
+    <definedName name="A128477400L_Latest">Data1!$AS$107</definedName>
+    <definedName name="A128477405X">Data1!$F$1:$F$10,Data1!$F$11:$F$107</definedName>
+    <definedName name="A128477405X_Data">Data1!$F$11:$F$107</definedName>
+    <definedName name="A128477405X_Latest">Data1!$F$107</definedName>
+    <definedName name="A128477406A">Data1!$AO$1:$AO$10,Data1!$AO$23:$AO$107</definedName>
+    <definedName name="A128477406A_Data">Data1!$AO$23:$AO$107</definedName>
+    <definedName name="A128477406A_Latest">Data1!$AO$107</definedName>
+    <definedName name="A128478317T">Data1!$B$1:$B$10,Data1!$B$11:$B$107</definedName>
+    <definedName name="A128478317T_Data">Data1!$B$11:$B$107</definedName>
+    <definedName name="A128478317T_Latest">Data1!$B$107</definedName>
+    <definedName name="A128478318V">Data1!$AK$1:$AK$10,Data1!$AK$23:$AK$107</definedName>
+    <definedName name="A128478318V_Data">Data1!$AK$23:$AK$107</definedName>
+    <definedName name="A128478318V_Latest">Data1!$AK$107</definedName>
+    <definedName name="A128478473V">Data1!$Y$1:$Y$10,Data1!$Y$11:$Y$107</definedName>
+    <definedName name="A128478473V_Data">Data1!$Y$11:$Y$107</definedName>
+    <definedName name="A128478473V_Latest">Data1!$Y$107</definedName>
+    <definedName name="A128478474W">Data1!$BH$1:$BH$10,Data1!$BH$23:$BH$107</definedName>
+    <definedName name="A128478474W_Data">Data1!$BH$23:$BH$107</definedName>
+    <definedName name="A128478474W_Latest">Data1!$BH$107</definedName>
+    <definedName name="A128478847A">Data1!$N$1:$N$10,Data1!$N$11:$N$107</definedName>
+    <definedName name="A128478847A_Data">Data1!$N$11:$N$107</definedName>
+    <definedName name="A128478847A_Latest">Data1!$N$107</definedName>
+    <definedName name="A128478848C">Data1!$AW$1:$AW$10,Data1!$AW$23:$AW$107</definedName>
+    <definedName name="A128478848C_Data">Data1!$AW$23:$AW$107</definedName>
+    <definedName name="A128478848C_Latest">Data1!$AW$107</definedName>
+    <definedName name="A128479215W">Data1!$E$1:$E$10,Data1!$E$11:$E$107</definedName>
+    <definedName name="A128479215W_Data">Data1!$E$11:$E$107</definedName>
+    <definedName name="A128479215W_Latest">Data1!$E$107</definedName>
+    <definedName name="A128479216X">Data1!$AN$1:$AN$10,Data1!$AN$23:$AN$107</definedName>
+    <definedName name="A128479216X_Data">Data1!$AN$23:$AN$107</definedName>
+    <definedName name="A128479216X_Latest">Data1!$AN$107</definedName>
+    <definedName name="A128479281V">Data1!$K$1:$K$10,Data1!$K$11:$K$107</definedName>
+    <definedName name="A128479281V_Data">Data1!$K$11:$K$107</definedName>
+    <definedName name="A128479281V_Latest">Data1!$K$107</definedName>
+    <definedName name="A128479282W">Data1!$AT$1:$AT$10,Data1!$AT$23:$AT$107</definedName>
+    <definedName name="A128479282W_Data">Data1!$AT$23:$AT$107</definedName>
+    <definedName name="A128479282W_Latest">Data1!$AT$107</definedName>
+    <definedName name="A128480133R">Data1!$AJ$1:$AJ$10,Data1!$AJ$11:$AJ$107</definedName>
+    <definedName name="A128480133R_Data">Data1!$AJ$11:$AJ$107</definedName>
+    <definedName name="A128480133R_Latest">Data1!$AJ$107</definedName>
+    <definedName name="A128480134T">Data1!$BT$1:$BT$10,Data1!$BT$23:$BT$107</definedName>
+    <definedName name="A128480134T_Data">Data1!$BT$23:$BT$107</definedName>
+    <definedName name="A128480134T_Latest">Data1!$BT$107</definedName>
+    <definedName name="A128480215V">Data1!$G$1:$G$10,Data1!$G$11:$G$107</definedName>
+    <definedName name="A128480215V_Data">Data1!$G$11:$G$107</definedName>
+    <definedName name="A128480215V_Latest">Data1!$G$107</definedName>
+    <definedName name="A128480216W">Data1!$AP$1:$AP$10,Data1!$AP$23:$AP$107</definedName>
+    <definedName name="A128480216W_Data">Data1!$AP$23:$AP$107</definedName>
+    <definedName name="A128480216W_Latest">Data1!$AP$107</definedName>
+    <definedName name="A128480733V">Data1!$C$1:$C$10,Data1!$C$11:$C$107</definedName>
+    <definedName name="A128480733V_Data">Data1!$C$11:$C$107</definedName>
+    <definedName name="A128480733V_Latest">Data1!$C$107</definedName>
+    <definedName name="A128480734W">Data1!$AL$1:$AL$10,Data1!$AL$23:$AL$107</definedName>
+    <definedName name="A128480734W_Data">Data1!$AL$23:$AL$107</definedName>
+    <definedName name="A128480734W_Latest">Data1!$AL$107</definedName>
+    <definedName name="A128481587A">Data1!$AD$1:$AD$10,Data1!$AD$11:$AD$107</definedName>
+    <definedName name="A128481587A_Data">Data1!$AD$11:$AD$107</definedName>
+    <definedName name="A128481587A_Latest">Data1!$AD$107</definedName>
+    <definedName name="A128481588C">Data1!$BM$1:$BM$10,Data1!$BM$23:$BM$107</definedName>
+    <definedName name="A128481588C_Data">Data1!$BM$23:$BM$107</definedName>
+    <definedName name="A128481588C_Latest">Data1!$BM$107</definedName>
+    <definedName name="A128481639T">Data1!$AH$1:$AH$10,Data1!$AH$11:$AH$107</definedName>
+    <definedName name="A128481639T_Data">Data1!$AH$11:$AH$107</definedName>
+    <definedName name="A128481639T_Latest">Data1!$AH$107</definedName>
+    <definedName name="A128481640A">Data1!$BR$1:$BR$10,Data1!$BR$23:$BR$107</definedName>
+    <definedName name="A128481640A_Data">Data1!$BR$23:$BR$107</definedName>
+    <definedName name="A128481640A_Latest">Data1!$BR$107</definedName>
+    <definedName name="A128482435J">Data1!$V$1:$V$10,Data1!$V$11:$V$107</definedName>
+    <definedName name="A128482435J_Data">Data1!$V$11:$V$107</definedName>
+    <definedName name="A128482435J_Latest">Data1!$V$107</definedName>
+    <definedName name="A128482436K">Data1!$BE$1:$BE$10,Data1!$BE$23:$BE$107</definedName>
+    <definedName name="A128482436K_Data">Data1!$BE$23:$BE$107</definedName>
+    <definedName name="A128482436K_Latest">Data1!$BE$107</definedName>
+    <definedName name="A128483461F">Data1!$AG$1:$AG$10,Data1!$AG$11:$AG$107</definedName>
+    <definedName name="A128483461F_Data">Data1!$AG$11:$AG$107</definedName>
+    <definedName name="A128483461F_Latest">Data1!$AG$107</definedName>
+    <definedName name="A128483462J">Data1!$BQ$1:$BQ$10,Data1!$BQ$23:$BQ$107</definedName>
+    <definedName name="A128483462J_Data">Data1!$BQ$23:$BQ$107</definedName>
+    <definedName name="A128483462J_Latest">Data1!$BQ$107</definedName>
+    <definedName name="A128484257R">Data1!$L$1:$L$10,Data1!$L$11:$L$107</definedName>
+    <definedName name="A128484257R_Data">Data1!$L$11:$L$107</definedName>
+    <definedName name="A128484257R_Latest">Data1!$L$107</definedName>
+    <definedName name="A128484258T">Data1!$AU$1:$AU$10,Data1!$AU$23:$AU$107</definedName>
+    <definedName name="A128484258T_Data">Data1!$AU$23:$AU$107</definedName>
+    <definedName name="A128484258T_Latest">Data1!$AU$107</definedName>
+    <definedName name="A128484685K">Data1!$W$1:$W$10,Data1!$W$11:$W$107</definedName>
+    <definedName name="A128484685K_Data">Data1!$W$11:$W$107</definedName>
+    <definedName name="A128484685K_Latest">Data1!$W$107</definedName>
+    <definedName name="A128484686L">Data1!$BF$1:$BF$10,Data1!$BF$23:$BF$107</definedName>
+    <definedName name="A128484686L_Data">Data1!$BF$23:$BF$107</definedName>
+    <definedName name="A128484686L_Latest">Data1!$BF$107</definedName>
+    <definedName name="A128485865L">Data1!$O$1:$O$10,Data1!$O$11:$O$107</definedName>
+    <definedName name="A128485865L_Data">Data1!$O$11:$O$107</definedName>
+    <definedName name="A128485865L_Latest">Data1!$O$107</definedName>
+    <definedName name="A128485866R">Data1!$AX$1:$AX$10,Data1!$AX$23:$AX$107</definedName>
+    <definedName name="A128485866R_Data">Data1!$AX$23:$AX$107</definedName>
+    <definedName name="A128485866R_Latest">Data1!$AX$107</definedName>
+    <definedName name="A128485881L">Data1!$T$1:$T$10,Data1!$T$11:$T$107</definedName>
+    <definedName name="A128485881L_Data">Data1!$T$11:$T$107</definedName>
+    <definedName name="A128485881L_Latest">Data1!$T$107</definedName>
+    <definedName name="A128485882R">Data1!$BC$1:$BC$10,Data1!$BC$23:$BC$107</definedName>
+    <definedName name="A128485882R_Data">Data1!$BC$23:$BC$107</definedName>
+    <definedName name="A128485882R_Latest">Data1!$BC$107</definedName>
+    <definedName name="A130184496J">Data1!$BN$1:$BN$10,Data1!$BN$23:$BN$107</definedName>
+    <definedName name="A130184496J_Data">Data1!$BN$23:$BN$107</definedName>
+    <definedName name="A130184496J_Latest">Data1!$BN$107</definedName>
+    <definedName name="A130184497K">Data1!$BP$1:$BP$10,Data1!$BP$23:$BP$107</definedName>
+    <definedName name="A130184497K_Data">Data1!$BP$23:$BP$107</definedName>
+    <definedName name="A130184497K_Latest">Data1!$BP$107</definedName>
+    <definedName name="A130184498L">Data1!$BO$1:$BO$10,Data1!$BO$23:$BO$107</definedName>
+    <definedName name="A130184498L_Data">Data1!$BO$23:$BO$107</definedName>
+    <definedName name="A130184498L_Latest">Data1!$BO$107</definedName>
+    <definedName name="A130184499R">Data1!$AE$1:$AE$10,Data1!$AE$11:$AE$107</definedName>
+    <definedName name="A130184499R_Data">Data1!$AE$11:$AE$107</definedName>
+    <definedName name="A130184499R_Latest">Data1!$AE$107</definedName>
+    <definedName name="A130184501R">Data1!$AF$1:$AF$10,Data1!$AF$11:$AF$107</definedName>
+    <definedName name="A130184501R_Data">Data1!$AF$11:$AF$107</definedName>
+    <definedName name="A130184501R_Latest">Data1!$AF$107</definedName>
+    <definedName name="Date_Range">Data1!$A$2:$A$10,Data1!$A$11:$A$107</definedName>
+    <definedName name="Date_Range_Data">Data1!$A$11:$A$107</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -1196,7 +1196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF24" authorId="0" shapeId="0">
+    <comment ref="AF18" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1209,59 +1209,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BO24" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BO36" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AF55" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BO55" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BO67" authorId="0" shapeId="0">
+    <comment ref="BO30" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1313,6 +1261,97 @@
         </r>
       </text>
     </comment>
+    <comment ref="AF86" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>revised</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="BO86" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>revised</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF94" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>revised</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="BO94" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>revised</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD97" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>revised</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="BM97" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>revised</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="BO98" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>revised</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="AD99" authorId="0" shapeId="0">
       <text>
         <r>
@@ -1339,59 +1378,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD102" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BM102" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AF103" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BO103" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>revised</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AD104" authorId="0" shapeId="0">
+    <comment ref="BO106" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -2587,10 +2574,10 @@
         <v>42979</v>
       </c>
       <c r="G12" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H12" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I12" s="10" t="s">
         <v>78</v>
@@ -2619,10 +2606,10 @@
         <v>42979</v>
       </c>
       <c r="G13" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H13" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I13" s="10" t="s">
         <v>78</v>
@@ -2651,10 +2638,10 @@
         <v>42979</v>
       </c>
       <c r="G14" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H14" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I14" s="10" t="s">
         <v>78</v>
@@ -2683,10 +2670,10 @@
         <v>42979</v>
       </c>
       <c r="G15" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H15" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>78</v>
@@ -2715,10 +2702,10 @@
         <v>42979</v>
       </c>
       <c r="G16" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H16" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>78</v>
@@ -2747,10 +2734,10 @@
         <v>42979</v>
       </c>
       <c r="G17" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H17" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>78</v>
@@ -2779,10 +2766,10 @@
         <v>42979</v>
       </c>
       <c r="G18" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H18" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>78</v>
@@ -2811,10 +2798,10 @@
         <v>42979</v>
       </c>
       <c r="G19" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H19" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I19" s="10" t="s">
         <v>78</v>
@@ -2843,10 +2830,10 @@
         <v>42979</v>
       </c>
       <c r="G20" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H20" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I20" s="10" t="s">
         <v>78</v>
@@ -2875,10 +2862,10 @@
         <v>42979</v>
       </c>
       <c r="G21" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H21" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>78</v>
@@ -2907,10 +2894,10 @@
         <v>42979</v>
       </c>
       <c r="G22" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H22" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>78</v>
@@ -2939,10 +2926,10 @@
         <v>42979</v>
       </c>
       <c r="G23" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H23" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>78</v>
@@ -2971,10 +2958,10 @@
         <v>42979</v>
       </c>
       <c r="G24" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H24" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>78</v>
@@ -3003,10 +2990,10 @@
         <v>42979</v>
       </c>
       <c r="G25" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H25" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>78</v>
@@ -3035,10 +3022,10 @@
         <v>42979</v>
       </c>
       <c r="G26" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H26" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>78</v>
@@ -3067,10 +3054,10 @@
         <v>42979</v>
       </c>
       <c r="G27" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H27" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>78</v>
@@ -3099,10 +3086,10 @@
         <v>42979</v>
       </c>
       <c r="G28" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H28" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>78</v>
@@ -3131,10 +3118,10 @@
         <v>42979</v>
       </c>
       <c r="G29" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H29" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I29" s="10" t="s">
         <v>78</v>
@@ -3163,10 +3150,10 @@
         <v>42979</v>
       </c>
       <c r="G30" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H30" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I30" s="10" t="s">
         <v>78</v>
@@ -3195,10 +3182,10 @@
         <v>42979</v>
       </c>
       <c r="G31" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H31" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I31" s="10" t="s">
         <v>78</v>
@@ -3227,10 +3214,10 @@
         <v>42979</v>
       </c>
       <c r="G32" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H32" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I32" s="10" t="s">
         <v>78</v>
@@ -3259,10 +3246,10 @@
         <v>42979</v>
       </c>
       <c r="G33" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H33" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I33" s="10" t="s">
         <v>78</v>
@@ -3291,10 +3278,10 @@
         <v>42979</v>
       </c>
       <c r="G34" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H34" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I34" s="10" t="s">
         <v>78</v>
@@ -3323,10 +3310,10 @@
         <v>42979</v>
       </c>
       <c r="G35" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H35" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I35" s="10" t="s">
         <v>78</v>
@@ -3355,10 +3342,10 @@
         <v>42979</v>
       </c>
       <c r="G36" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H36" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I36" s="10" t="s">
         <v>78</v>
@@ -3387,10 +3374,10 @@
         <v>42979</v>
       </c>
       <c r="G37" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H37" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I37" s="10" t="s">
         <v>78</v>
@@ -3419,10 +3406,10 @@
         <v>42979</v>
       </c>
       <c r="G38" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H38" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I38" s="10" t="s">
         <v>78</v>
@@ -3451,10 +3438,10 @@
         <v>42979</v>
       </c>
       <c r="G39" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H39" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I39" s="10" t="s">
         <v>78</v>
@@ -3483,10 +3470,10 @@
         <v>42979</v>
       </c>
       <c r="G40" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H40" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I40" s="10" t="s">
         <v>78</v>
@@ -3515,10 +3502,10 @@
         <v>42979</v>
       </c>
       <c r="G41" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H41" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I41" s="10" t="s">
         <v>78</v>
@@ -3547,10 +3534,10 @@
         <v>42979</v>
       </c>
       <c r="G42" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H42" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I42" s="10" t="s">
         <v>78</v>
@@ -3579,10 +3566,10 @@
         <v>42979</v>
       </c>
       <c r="G43" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H43" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I43" s="10" t="s">
         <v>78</v>
@@ -3611,10 +3598,10 @@
         <v>42979</v>
       </c>
       <c r="G44" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H44" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I44" s="10" t="s">
         <v>78</v>
@@ -3643,10 +3630,10 @@
         <v>42979</v>
       </c>
       <c r="G45" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H45" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I45" s="10" t="s">
         <v>78</v>
@@ -3675,10 +3662,10 @@
         <v>42979</v>
       </c>
       <c r="G46" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H46" s="10">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I46" s="10" t="s">
         <v>78</v>
@@ -3707,10 +3694,10 @@
         <v>43344</v>
       </c>
       <c r="G47" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H47" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I47" s="10" t="s">
         <v>118</v>
@@ -3739,10 +3726,10 @@
         <v>43344</v>
       </c>
       <c r="G48" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H48" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I48" s="10" t="s">
         <v>118</v>
@@ -3771,10 +3758,10 @@
         <v>43344</v>
       </c>
       <c r="G49" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H49" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I49" s="10" t="s">
         <v>118</v>
@@ -3803,10 +3790,10 @@
         <v>43344</v>
       </c>
       <c r="G50" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H50" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I50" s="10" t="s">
         <v>118</v>
@@ -3835,10 +3822,10 @@
         <v>43344</v>
       </c>
       <c r="G51" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H51" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I51" s="10" t="s">
         <v>118</v>
@@ -3867,10 +3854,10 @@
         <v>43344</v>
       </c>
       <c r="G52" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H52" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I52" s="10" t="s">
         <v>118</v>
@@ -3899,10 +3886,10 @@
         <v>43344</v>
       </c>
       <c r="G53" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H53" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>118</v>
@@ -3931,10 +3918,10 @@
         <v>43344</v>
       </c>
       <c r="G54" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H54" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I54" s="10" t="s">
         <v>118</v>
@@ -3963,10 +3950,10 @@
         <v>43344</v>
       </c>
       <c r="G55" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H55" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I55" s="10" t="s">
         <v>118</v>
@@ -3995,10 +3982,10 @@
         <v>43344</v>
       </c>
       <c r="G56" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H56" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I56" s="10" t="s">
         <v>118</v>
@@ -4027,10 +4014,10 @@
         <v>43344</v>
       </c>
       <c r="G57" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H57" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I57" s="10" t="s">
         <v>118</v>
@@ -4059,10 +4046,10 @@
         <v>43344</v>
       </c>
       <c r="G58" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H58" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I58" s="10" t="s">
         <v>118</v>
@@ -4091,10 +4078,10 @@
         <v>43344</v>
       </c>
       <c r="G59" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H59" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I59" s="10" t="s">
         <v>118</v>
@@ -4123,10 +4110,10 @@
         <v>43344</v>
       </c>
       <c r="G60" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H60" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I60" s="10" t="s">
         <v>118</v>
@@ -4155,10 +4142,10 @@
         <v>43344</v>
       </c>
       <c r="G61" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H61" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I61" s="10" t="s">
         <v>118</v>
@@ -4187,10 +4174,10 @@
         <v>43344</v>
       </c>
       <c r="G62" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H62" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I62" s="10" t="s">
         <v>118</v>
@@ -4219,10 +4206,10 @@
         <v>43344</v>
       </c>
       <c r="G63" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H63" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I63" s="10" t="s">
         <v>118</v>
@@ -4251,10 +4238,10 @@
         <v>43344</v>
       </c>
       <c r="G64" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H64" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I64" s="10" t="s">
         <v>118</v>
@@ -4283,10 +4270,10 @@
         <v>43344</v>
       </c>
       <c r="G65" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H65" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I65" s="10" t="s">
         <v>118</v>
@@ -4315,10 +4302,10 @@
         <v>43344</v>
       </c>
       <c r="G66" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H66" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I66" s="10" t="s">
         <v>118</v>
@@ -4347,10 +4334,10 @@
         <v>43344</v>
       </c>
       <c r="G67" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H67" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I67" s="10" t="s">
         <v>118</v>
@@ -4379,10 +4366,10 @@
         <v>43344</v>
       </c>
       <c r="G68" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H68" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I68" s="10" t="s">
         <v>118</v>
@@ -4411,10 +4398,10 @@
         <v>43344</v>
       </c>
       <c r="G69" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H69" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I69" s="10" t="s">
         <v>118</v>
@@ -4443,10 +4430,10 @@
         <v>43344</v>
       </c>
       <c r="G70" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H70" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I70" s="10" t="s">
         <v>118</v>
@@ -4475,10 +4462,10 @@
         <v>43344</v>
       </c>
       <c r="G71" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H71" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I71" s="10" t="s">
         <v>118</v>
@@ -4507,10 +4494,10 @@
         <v>43344</v>
       </c>
       <c r="G72" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H72" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I72" s="10" t="s">
         <v>118</v>
@@ -4539,10 +4526,10 @@
         <v>43344</v>
       </c>
       <c r="G73" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H73" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I73" s="10" t="s">
         <v>118</v>
@@ -4571,10 +4558,10 @@
         <v>43344</v>
       </c>
       <c r="G74" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H74" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I74" s="10" t="s">
         <v>118</v>
@@ -4603,10 +4590,10 @@
         <v>43344</v>
       </c>
       <c r="G75" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H75" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I75" s="10" t="s">
         <v>118</v>
@@ -4635,10 +4622,10 @@
         <v>43344</v>
       </c>
       <c r="G76" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H76" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I76" s="10" t="s">
         <v>118</v>
@@ -4667,10 +4654,10 @@
         <v>43344</v>
       </c>
       <c r="G77" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H77" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I77" s="10" t="s">
         <v>118</v>
@@ -4699,10 +4686,10 @@
         <v>43344</v>
       </c>
       <c r="G78" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H78" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I78" s="10" t="s">
         <v>118</v>
@@ -4731,10 +4718,10 @@
         <v>43344</v>
       </c>
       <c r="G79" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H79" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I79" s="10" t="s">
         <v>118</v>
@@ -4763,10 +4750,10 @@
         <v>43344</v>
       </c>
       <c r="G80" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H80" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I80" s="10" t="s">
         <v>118</v>
@@ -4795,10 +4782,10 @@
         <v>43344</v>
       </c>
       <c r="G81" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H81" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I81" s="10" t="s">
         <v>118</v>
@@ -4827,10 +4814,10 @@
         <v>43344</v>
       </c>
       <c r="G82" s="9">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H82" s="10">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I82" s="10" t="s">
         <v>118</v>
@@ -4936,7 +4923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BT105"/>
+  <dimension ref="A1:BT107"/>
   <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="14.7109375" style="1"/>
@@ -6470,217 +6457,217 @@
         <v>75</v>
       </c>
       <c r="B8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="C8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="D8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="E8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="F8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="G8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="H8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="I8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="J8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="K8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="L8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="M8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="N8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="O8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="P8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="Q8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="R8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="S8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="T8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="U8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="V8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="W8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="X8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="Y8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="Z8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AA8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AB8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AC8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AD8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AE8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AF8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AG8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AH8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AI8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AJ8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AK8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AL8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AM8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AN8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AO8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AP8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AQ8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AR8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AS8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AT8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AU8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AV8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AW8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AX8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AY8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="AZ8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BA8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BB8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BC8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BD8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BE8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BF8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BG8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BH8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BI8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BJ8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BK8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BL8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BM8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BN8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BO8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BP8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BQ8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BR8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BS8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
       <c r="BT8" s="6">
-        <v>45839</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="9" spans="1:72" x14ac:dyDescent="0.2">
@@ -6688,217 +6675,217 @@
         <v>76</v>
       </c>
       <c r="B9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="N9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="O9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="P9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="Q9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="S9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="T9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="U9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="V9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="W9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="X9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="Y9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="Z9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AA9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AB9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AC9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AD9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AE9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AF9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AG9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AH9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AI9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AJ9" s="1">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AK9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AL9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AM9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AN9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AO9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AP9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AQ9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AR9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AS9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AT9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AU9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AV9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AW9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AX9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AY9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AZ9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BA9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BB9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BC9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BD9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BE9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BF9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BG9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BH9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BI9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BJ9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BK9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BL9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BM9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BN9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BO9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BP9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BQ9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BR9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BS9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="BT9" s="1">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:72" x14ac:dyDescent="0.2">
@@ -7984,7 +7971,7 @@
         <v>101</v>
       </c>
       <c r="AF18" s="8">
-        <v>100.8</v>
+        <v>100.7</v>
       </c>
       <c r="AG18" s="8">
         <v>101.7</v>
@@ -10165,7 +10152,7 @@
         <v>1.4</v>
       </c>
       <c r="BO30" s="8">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="BP30" s="8">
         <v>1.6</v>
@@ -18780,7 +18767,7 @@
         <v>113.7</v>
       </c>
       <c r="AF70" s="8">
-        <v>113.7</v>
+        <v>113.8</v>
       </c>
       <c r="AG70" s="8">
         <v>119.4</v>
@@ -18885,7 +18872,7 @@
         <v>6.6</v>
       </c>
       <c r="BO70" s="8">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="BP70" s="8">
         <v>5.9</v>
@@ -21501,7 +21488,7 @@
         <v>5.5</v>
       </c>
       <c r="BO82" s="8">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="BP82" s="8">
         <v>5.6</v>
@@ -21614,7 +21601,7 @@
         <v>120.4</v>
       </c>
       <c r="AF83" s="8">
-        <v>120.4</v>
+        <v>120.3</v>
       </c>
       <c r="AG83" s="8">
         <v>126.1</v>
@@ -21719,7 +21706,7 @@
         <v>5.5</v>
       </c>
       <c r="BO83" s="8">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="BP83" s="8">
         <v>5.4</v>
@@ -22268,7 +22255,7 @@
         <v>121</v>
       </c>
       <c r="AF86" s="8">
-        <v>121.2</v>
+        <v>121.1</v>
       </c>
       <c r="AG86" s="8">
         <v>125.7</v>
@@ -22373,7 +22360,7 @@
         <v>4.2</v>
       </c>
       <c r="BO86" s="8">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="BP86" s="8">
         <v>4</v>
@@ -24335,7 +24322,7 @@
         <v>2.7</v>
       </c>
       <c r="BO95" s="8">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="BP95" s="8">
         <v>3.2</v>
@@ -24660,7 +24647,7 @@
         <v>123.3</v>
       </c>
       <c r="AD97" s="8">
-        <v>124.8</v>
+        <v>124.7</v>
       </c>
       <c r="AE97" s="8">
         <v>124.3</v>
@@ -24765,7 +24752,7 @@
         <v>2.7</v>
       </c>
       <c r="BM97" s="8">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="BN97" s="8">
         <v>2.8</v>
@@ -24989,7 +24976,7 @@
         <v>2.7</v>
       </c>
       <c r="BO98" s="8">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="BP98" s="8">
         <v>2.7</v>
@@ -25096,7 +25083,7 @@
         <v>123.9</v>
       </c>
       <c r="AD99" s="8">
-        <v>125.6</v>
+        <v>125.5</v>
       </c>
       <c r="AE99" s="8">
         <v>124.5</v>
@@ -25201,7 +25188,7 @@
         <v>2.7</v>
       </c>
       <c r="BM99" s="8">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="BN99" s="8">
         <v>2.9</v>
@@ -26368,7 +26355,7 @@
         <v>142.80000000000001</v>
       </c>
       <c r="R105" s="8">
-        <v>118.8</v>
+        <v>119.3</v>
       </c>
       <c r="S105" s="8">
         <v>145.6</v>
@@ -26410,7 +26397,7 @@
         <v>127.6</v>
       </c>
       <c r="AF105" s="8">
-        <v>127.6</v>
+        <v>127.7</v>
       </c>
       <c r="AG105" s="8">
         <v>130.80000000000001</v>
@@ -26473,7 +26460,7 @@
         <v>0.4</v>
       </c>
       <c r="BA105" s="8">
-        <v>13.1</v>
+        <v>13.6</v>
       </c>
       <c r="BB105" s="8">
         <v>4.7</v>
@@ -26515,7 +26502,7 @@
         <v>3.2</v>
       </c>
       <c r="BO105" s="8">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="BP105" s="8">
         <v>2.7</v>
@@ -26531,6 +26518,442 @@
       </c>
       <c r="BT105" s="8">
         <v>3.9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:72" x14ac:dyDescent="0.2">
+      <c r="A106" s="9">
+        <v>45870</v>
+      </c>
+      <c r="B106" s="8">
+        <v>127.6</v>
+      </c>
+      <c r="C106" s="8">
+        <v>134.6</v>
+      </c>
+      <c r="D106" s="8">
+        <v>136.6</v>
+      </c>
+      <c r="E106" s="8">
+        <v>131.6</v>
+      </c>
+      <c r="F106" s="8">
+        <v>138</v>
+      </c>
+      <c r="G106" s="8">
+        <v>144.9</v>
+      </c>
+      <c r="H106" s="8">
+        <v>135.19999999999999</v>
+      </c>
+      <c r="I106" s="8">
+        <v>138.1</v>
+      </c>
+      <c r="J106" s="8">
+        <v>155</v>
+      </c>
+      <c r="K106" s="8">
+        <v>121.9</v>
+      </c>
+      <c r="L106" s="8">
+        <v>224.9</v>
+      </c>
+      <c r="M106" s="8">
+        <v>107.6</v>
+      </c>
+      <c r="N106" s="8">
+        <v>102.7</v>
+      </c>
+      <c r="O106" s="8">
+        <v>130.19999999999999</v>
+      </c>
+      <c r="P106" s="8">
+        <v>122</v>
+      </c>
+      <c r="Q106" s="8">
+        <v>143.4</v>
+      </c>
+      <c r="R106" s="8">
+        <v>111.8</v>
+      </c>
+      <c r="S106" s="8">
+        <v>145.9</v>
+      </c>
+      <c r="T106" s="8">
+        <v>118.9</v>
+      </c>
+      <c r="U106" s="8">
+        <v>133.19999999999999</v>
+      </c>
+      <c r="V106" s="8">
+        <v>130.5</v>
+      </c>
+      <c r="W106" s="8">
+        <v>144.30000000000001</v>
+      </c>
+      <c r="X106" s="8">
+        <v>92.2</v>
+      </c>
+      <c r="Y106" s="8">
+        <v>112.3</v>
+      </c>
+      <c r="Z106" s="8">
+        <v>116.7</v>
+      </c>
+      <c r="AA106" s="8">
+        <v>133.19999999999999</v>
+      </c>
+      <c r="AB106" s="8">
+        <v>128.6</v>
+      </c>
+      <c r="AC106" s="8">
+        <v>126.7</v>
+      </c>
+      <c r="AD106" s="8">
+        <v>128</v>
+      </c>
+      <c r="AE106" s="8">
+        <v>127.8</v>
+      </c>
+      <c r="AF106" s="8">
+        <v>127.8</v>
+      </c>
+      <c r="AG106" s="8">
+        <v>130.80000000000001</v>
+      </c>
+      <c r="AH106" s="8">
+        <v>123.6</v>
+      </c>
+      <c r="AI106" s="8">
+        <v>119.8</v>
+      </c>
+      <c r="AJ106" s="8">
+        <v>131.9</v>
+      </c>
+      <c r="AK106" s="8">
+        <v>3</v>
+      </c>
+      <c r="AL106" s="8">
+        <v>3</v>
+      </c>
+      <c r="AM106" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="AN106" s="8">
+        <v>2.9</v>
+      </c>
+      <c r="AO106" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="AP106" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AQ106" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AR106" s="8">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="AS106" s="8">
+        <v>6</v>
+      </c>
+      <c r="AT106" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="AU106" s="8">
+        <v>12.6</v>
+      </c>
+      <c r="AV106" s="8">
+        <v>3</v>
+      </c>
+      <c r="AW106" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="AX106" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="AY106" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="AZ106" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="BA106" s="8">
+        <v>24.6</v>
+      </c>
+      <c r="BB106" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="BC106" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="BD106" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="BE106" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="BF106" s="8">
+        <v>-1.7</v>
+      </c>
+      <c r="BG106" s="8">
+        <v>1.9</v>
+      </c>
+      <c r="BH106" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="BI106" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="BJ106" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="BK106" s="8">
+        <v>3</v>
+      </c>
+      <c r="BL106" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="BM106" s="8">
+        <v>3</v>
+      </c>
+      <c r="BN106" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="BO106" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="BP106" s="8">
+        <v>2.6</v>
+      </c>
+      <c r="BQ106" s="8">
+        <v>2.8</v>
+      </c>
+      <c r="BR106" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="BS106" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="BT106" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="107" spans="1:72" x14ac:dyDescent="0.2">
+      <c r="A107" s="9">
+        <v>45901</v>
+      </c>
+      <c r="B107" s="8">
+        <v>128.30000000000001</v>
+      </c>
+      <c r="C107" s="8">
+        <v>134</v>
+      </c>
+      <c r="D107" s="8">
+        <v>136.19999999999999</v>
+      </c>
+      <c r="E107" s="8">
+        <v>132.19999999999999</v>
+      </c>
+      <c r="F107" s="8">
+        <v>139</v>
+      </c>
+      <c r="G107" s="8">
+        <v>139.1</v>
+      </c>
+      <c r="H107" s="8">
+        <v>136</v>
+      </c>
+      <c r="I107" s="8">
+        <v>137</v>
+      </c>
+      <c r="J107" s="8">
+        <v>156.80000000000001</v>
+      </c>
+      <c r="K107" s="8">
+        <v>121.3</v>
+      </c>
+      <c r="L107" s="8">
+        <v>236.6</v>
+      </c>
+      <c r="M107" s="8">
+        <v>106.5</v>
+      </c>
+      <c r="N107" s="8">
+        <v>100.9</v>
+      </c>
+      <c r="O107" s="8">
+        <v>131.4</v>
+      </c>
+      <c r="P107" s="8">
+        <v>122.3</v>
+      </c>
+      <c r="Q107" s="8">
+        <v>144.4</v>
+      </c>
+      <c r="R107" s="8">
+        <v>111.3</v>
+      </c>
+      <c r="S107" s="8">
+        <v>149.30000000000001</v>
+      </c>
+      <c r="T107" s="8">
+        <v>119.2</v>
+      </c>
+      <c r="U107" s="8">
+        <v>133.19999999999999</v>
+      </c>
+      <c r="V107" s="8">
+        <v>131</v>
+      </c>
+      <c r="W107" s="8">
+        <v>145</v>
+      </c>
+      <c r="X107" s="8">
+        <v>92</v>
+      </c>
+      <c r="Y107" s="8">
+        <v>115</v>
+      </c>
+      <c r="Z107" s="8">
+        <v>122.3</v>
+      </c>
+      <c r="AA107" s="8">
+        <v>133.30000000000001</v>
+      </c>
+      <c r="AB107" s="8">
+        <v>128.9</v>
+      </c>
+      <c r="AC107" s="8">
+        <v>127.5</v>
+      </c>
+      <c r="AD107" s="8">
+        <v>128.4</v>
+      </c>
+      <c r="AE107" s="8">
+        <v>128.30000000000001</v>
+      </c>
+      <c r="AF107" s="8">
+        <v>128.30000000000001</v>
+      </c>
+      <c r="AG107" s="8">
+        <v>131</v>
+      </c>
+      <c r="AH107" s="8">
+        <v>124.8</v>
+      </c>
+      <c r="AI107" s="8">
+        <v>120.1</v>
+      </c>
+      <c r="AJ107" s="8">
+        <v>132.80000000000001</v>
+      </c>
+      <c r="AK107" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="AL107" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="AM107" s="8">
+        <v>1.9</v>
+      </c>
+      <c r="AN107" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="AO107" s="8">
+        <v>2.6</v>
+      </c>
+      <c r="AP107" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="AQ107" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="AR107" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="AS107" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="AT107" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AU107" s="8">
+        <v>13.5</v>
+      </c>
+      <c r="AV107" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="AW107" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="AX107" s="8">
+        <v>5.6</v>
+      </c>
+      <c r="AY107" s="8">
+        <v>3.8</v>
+      </c>
+      <c r="AZ107" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="BA107" s="8">
+        <v>33.9</v>
+      </c>
+      <c r="BB107" s="8">
+        <v>6.4</v>
+      </c>
+      <c r="BC107" s="8">
+        <v>1</v>
+      </c>
+      <c r="BD107" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="BE107" s="8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="BF107" s="8">
+        <v>2.8</v>
+      </c>
+      <c r="BG107" s="8">
+        <v>1.9</v>
+      </c>
+      <c r="BH107" s="8">
+        <v>1.9</v>
+      </c>
+      <c r="BI107" s="8">
+        <v>1.9</v>
+      </c>
+      <c r="BJ107" s="8">
+        <v>5.3</v>
+      </c>
+      <c r="BK107" s="8">
+        <v>2.6</v>
+      </c>
+      <c r="BL107" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="BM107" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="BN107" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="BO107" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="BP107" s="8">
+        <v>2.8</v>
+      </c>
+      <c r="BQ107" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="BR107" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="BS107" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="BT107" s="8">
+        <v>4.4000000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>